<commit_message>
auto: add Li futures, fix yAxis scale
</commit_message>
<xml_diff>
--- a/金属价格日报.xlsx
+++ b/金属价格日报.xlsx
@@ -5674,14 +5674,14 @@
         </is>
       </c>
       <c r="D7" s="6" t="n">
-        <v>6.7614</v>
+        <v>6.7571</v>
       </c>
       <c r="E7" s="5" t="n"/>
       <c r="F7" s="6" t="n">
         <v>6.7621</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>6.7565</v>
+        <v>6.756</v>
       </c>
       <c r="H7" s="5" t="n"/>
       <c r="I7" s="5" t="inlineStr">
@@ -5712,13 +5712,13 @@
         </is>
       </c>
       <c r="D8" s="6" t="n">
-        <v>21.96</v>
+        <v>22.27</v>
       </c>
       <c r="E8" s="5" t="n"/>
       <c r="F8" s="5" t="n"/>
       <c r="G8" s="5" t="n"/>
-      <c r="H8" s="4" t="n">
-        <v>0</v>
+      <c r="H8" s="6" t="n">
+        <v>0.31</v>
       </c>
       <c r="I8" s="5" t="inlineStr">
         <is>

</xml_diff>